<commit_message>
Added functionality for bulk upload of faculty/staff details for registration
</commit_message>
<xml_diff>
--- a/backend/student_bulk_registration_template.xlsx
+++ b/backend/student_bulk_registration_template.xlsx
@@ -580,7 +580,7 @@
       <formula1>"Male,Female,Other,M,F,O"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Your entry is not in the list" type="list">
-      <formula1>"Student,Faculty,Staff,Dependent,Other"</formula1>
+      <formula1>"Student,Other"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -597,6 +597,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,9 +606,11 @@
           <t>BITS MED-C Bulk Registration Guide</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -615,20 +618,23 @@
           <t>1. DO NOT change the header names in the first row.</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. Fill student details starting from the second row.</t>
-        </is>
-      </c>
+          <t>2. Sample details have been provided in the first 2 rows. Fill student details starting from the third row.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Date of Birth must be in YYYY-MM-DD format.</t>
-        </is>
-      </c>
+          <t>3. Date of Birth must be in YYYY-MM-DD or DD-MM-YYYY format.</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -636,6 +642,7 @@
           <t>4. Gender and Patient Type have drop-down selections for accuracy.</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -643,6 +650,7 @@
           <t>5. Contact Number should be 10 digits without any spaces or country code.</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -650,9 +658,11 @@
           <t>6. IMPORTANT: When finished, go to File -&gt; Save As -&gt; Choose CSV (.csv) before uploading.</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -664,96 +674,96 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>institute_id</t>
+          <t>institute_id *</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bits ID / Institute ID (e.g., 2025H1120147P)</t>
+          <t>Bits ID / Institute ID (e.g., 2025H1120147P) (Mandatory)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>name *</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Full Name of the student</t>
+          <t>Full Name of the student (Mandatory)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>email *</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Official bits-pilani.ac.in email</t>
+          <t>Official bits-pilani.ac.in email (Mandatory)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>date_of_birth</t>
+          <t>date_of_birth *</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Format: YYYY-MM-DD</t>
+          <t>Format: YYYY-MM-DD or DD-MM-YYYY (Mandatory)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>gender *</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Select from drop-down or use M, F, O</t>
+          <t>Select from drop-down or use M, F, O (Mandatory)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>contact_no</t>
+          <t>contact_no *</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10-digit mobile number</t>
+          <t>10-digit mobile number (Mandatory)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>patient_type</t>
+          <t>patient_type *</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Select from drop-down</t>
+          <t>Select from drop-down (Mandatory)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>address</t>
+          <t>address *</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Hostel name or local address</t>
+          <t>Hostel name or local address (Mandatory)</t>
         </is>
       </c>
     </row>

</xml_diff>